<commit_message>
split logic and ui
</commit_message>
<xml_diff>
--- a/Design/config/HeroConfig.xlsx
+++ b/Design/config/HeroConfig.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2305" uniqueCount="988">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2305" uniqueCount="990">
   <si>
     <t>序列</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -3771,6 +3771,14 @@
   </si>
   <si>
     <t>死亡</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>弓</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>刀</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -3961,7 +3969,323 @@
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="179">
+  <dxfs count="219">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -6720,7 +7044,7 @@
         <v>1</v>
       </c>
       <c r="T14" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U14" s="5"/>
       <c r="V14" s="5"/>
@@ -6796,7 +7120,7 @@
         <v>1</v>
       </c>
       <c r="T15" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U15" s="5"/>
       <c r="V15" s="5"/>
@@ -6868,7 +7192,7 @@
         <v>1</v>
       </c>
       <c r="T16" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U16" s="5"/>
       <c r="V16" s="5"/>
@@ -6940,7 +7264,7 @@
         <v>1</v>
       </c>
       <c r="T17" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U17" s="5"/>
       <c r="V17" s="5"/>
@@ -8123,7 +8447,7 @@
         <v>3</v>
       </c>
       <c r="T32" s="5" t="s">
-        <v>292</v>
+        <v>988</v>
       </c>
       <c r="U32" s="5"/>
       <c r="V32" s="5"/>
@@ -9774,7 +10098,7 @@
         <v>1</v>
       </c>
       <c r="T53" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U53" s="5"/>
       <c r="V53" s="5"/>
@@ -9846,7 +10170,7 @@
         <v>1</v>
       </c>
       <c r="T54" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U54" s="5"/>
       <c r="V54" s="5"/>
@@ -9918,7 +10242,7 @@
         <v>1</v>
       </c>
       <c r="T55" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U55" s="5"/>
       <c r="V55" s="5"/>
@@ -9990,7 +10314,7 @@
         <v>1</v>
       </c>
       <c r="T56" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U56" s="5"/>
       <c r="V56" s="5"/>
@@ -10062,7 +10386,7 @@
         <v>1</v>
       </c>
       <c r="T57" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U57" s="5"/>
       <c r="V57" s="5"/>
@@ -10134,7 +10458,7 @@
         <v>1</v>
       </c>
       <c r="T58" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U58" s="5"/>
       <c r="V58" s="5"/>
@@ -10206,7 +10530,7 @@
         <v>1</v>
       </c>
       <c r="T59" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U59" s="5"/>
       <c r="V59" s="5"/>
@@ -10278,7 +10602,7 @@
         <v>1</v>
       </c>
       <c r="T60" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U60" s="5"/>
       <c r="V60" s="5"/>
@@ -10350,7 +10674,7 @@
         <v>1</v>
       </c>
       <c r="T61" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U61" s="5"/>
       <c r="V61" s="5"/>
@@ -10422,7 +10746,7 @@
         <v>1</v>
       </c>
       <c r="T62" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U62" s="5"/>
       <c r="V62" s="5"/>
@@ -10494,7 +10818,7 @@
         <v>1</v>
       </c>
       <c r="T63" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U63" s="5"/>
       <c r="V63" s="5"/>
@@ -10566,7 +10890,7 @@
         <v>1</v>
       </c>
       <c r="T64" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U64" s="5"/>
       <c r="V64" s="5"/>
@@ -10638,7 +10962,7 @@
         <v>1</v>
       </c>
       <c r="T65" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U65" s="5"/>
       <c r="V65" s="5"/>
@@ -10710,7 +11034,7 @@
         <v>1</v>
       </c>
       <c r="T66" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U66" s="5"/>
       <c r="V66" s="5"/>
@@ -10782,7 +11106,7 @@
         <v>1</v>
       </c>
       <c r="T67" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U67" s="5"/>
       <c r="V67" s="5"/>
@@ -10854,7 +11178,7 @@
         <v>1</v>
       </c>
       <c r="T68" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U68" s="5"/>
       <c r="V68" s="5"/>
@@ -10926,7 +11250,7 @@
         <v>1</v>
       </c>
       <c r="T69" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U69" s="5"/>
       <c r="V69" s="5"/>
@@ -10998,7 +11322,7 @@
         <v>1</v>
       </c>
       <c r="T70" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U70" s="5"/>
       <c r="V70" s="5"/>
@@ -11070,7 +11394,7 @@
         <v>1</v>
       </c>
       <c r="T71" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U71" s="5"/>
       <c r="V71" s="5"/>
@@ -11142,7 +11466,7 @@
         <v>1</v>
       </c>
       <c r="T72" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U72" s="5"/>
       <c r="V72" s="5"/>
@@ -11214,7 +11538,7 @@
         <v>1</v>
       </c>
       <c r="T73" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U73" s="5"/>
       <c r="V73" s="5"/>
@@ -11286,7 +11610,7 @@
         <v>1</v>
       </c>
       <c r="T74" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U74" s="5"/>
       <c r="V74" s="5"/>
@@ -11358,7 +11682,7 @@
         <v>1</v>
       </c>
       <c r="T75" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U75" s="5"/>
       <c r="V75" s="5"/>
@@ -11430,7 +11754,7 @@
         <v>1</v>
       </c>
       <c r="T76" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U76" s="5"/>
       <c r="V76" s="5"/>
@@ -11502,7 +11826,7 @@
         <v>1</v>
       </c>
       <c r="T77" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U77" s="5"/>
       <c r="V77" s="5"/>
@@ -11574,7 +11898,7 @@
         <v>1</v>
       </c>
       <c r="T78" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U78" s="5"/>
       <c r="V78" s="5"/>
@@ -11646,7 +11970,7 @@
         <v>1</v>
       </c>
       <c r="T79" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U79" s="5"/>
       <c r="V79" s="5"/>
@@ -11718,7 +12042,7 @@
         <v>1</v>
       </c>
       <c r="T80" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U80" s="5"/>
       <c r="V80" s="5"/>
@@ -11790,7 +12114,7 @@
         <v>1</v>
       </c>
       <c r="T81" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U81" s="5"/>
       <c r="V81" s="5"/>
@@ -11862,7 +12186,7 @@
         <v>1</v>
       </c>
       <c r="T82" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U82" s="5"/>
       <c r="V82" s="5"/>
@@ -11934,7 +12258,7 @@
         <v>1</v>
       </c>
       <c r="T83" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U83" s="5"/>
       <c r="V83" s="5"/>
@@ -12006,7 +12330,7 @@
         <v>1</v>
       </c>
       <c r="T84" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U84" s="5"/>
       <c r="V84" s="5"/>
@@ -12078,7 +12402,7 @@
         <v>1</v>
       </c>
       <c r="T85" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U85" s="5"/>
       <c r="V85" s="5"/>
@@ -12150,7 +12474,7 @@
         <v>1</v>
       </c>
       <c r="T86" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U86" s="5"/>
       <c r="V86" s="5"/>
@@ -14845,7 +15169,7 @@
         <v>1</v>
       </c>
       <c r="T120" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U120" s="5"/>
       <c r="V120" s="5"/>
@@ -14917,7 +15241,7 @@
         <v>1</v>
       </c>
       <c r="T121" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U121" s="5"/>
       <c r="V121" s="5"/>
@@ -14989,7 +15313,7 @@
         <v>1</v>
       </c>
       <c r="T122" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U122" s="5"/>
       <c r="V122" s="5"/>
@@ -15061,7 +15385,7 @@
         <v>1</v>
       </c>
       <c r="T123" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U123" s="5"/>
       <c r="V123" s="5"/>
@@ -15133,7 +15457,7 @@
         <v>1</v>
       </c>
       <c r="T124" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U124" s="5"/>
       <c r="V124" s="5"/>
@@ -15205,7 +15529,7 @@
         <v>1</v>
       </c>
       <c r="T125" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U125" s="5"/>
       <c r="V125" s="5"/>
@@ -15277,7 +15601,7 @@
         <v>1</v>
       </c>
       <c r="T126" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U126" s="5"/>
       <c r="V126" s="5"/>
@@ -15349,7 +15673,7 @@
         <v>1</v>
       </c>
       <c r="T127" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U127" s="5"/>
       <c r="V127" s="5"/>
@@ -15421,7 +15745,7 @@
         <v>1</v>
       </c>
       <c r="T128" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U128" s="5"/>
       <c r="V128" s="5"/>
@@ -15493,7 +15817,7 @@
         <v>1</v>
       </c>
       <c r="T129" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U129" s="5"/>
       <c r="V129" s="5"/>
@@ -15565,7 +15889,7 @@
         <v>1</v>
       </c>
       <c r="T130" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U130" s="5"/>
       <c r="V130" s="5"/>
@@ -15637,7 +15961,7 @@
         <v>1</v>
       </c>
       <c r="T131" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U131" s="5"/>
       <c r="V131" s="5"/>
@@ -15709,7 +16033,7 @@
         <v>1</v>
       </c>
       <c r="T132" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U132" s="5"/>
       <c r="V132" s="5"/>
@@ -15781,7 +16105,7 @@
         <v>1</v>
       </c>
       <c r="T133" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U133" s="5"/>
       <c r="V133" s="5"/>
@@ -15853,7 +16177,7 @@
         <v>1</v>
       </c>
       <c r="T134" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U134" s="5"/>
       <c r="V134" s="5"/>
@@ -15925,7 +16249,7 @@
         <v>1</v>
       </c>
       <c r="T135" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U135" s="5"/>
       <c r="V135" s="5"/>
@@ -15997,7 +16321,7 @@
         <v>1</v>
       </c>
       <c r="T136" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U136" s="5"/>
       <c r="V136" s="5"/>
@@ -16069,7 +16393,7 @@
         <v>1</v>
       </c>
       <c r="T137" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U137" s="5"/>
       <c r="V137" s="5"/>
@@ -16141,7 +16465,7 @@
         <v>1</v>
       </c>
       <c r="T138" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U138" s="5"/>
       <c r="V138" s="5"/>
@@ -16960,7 +17284,7 @@
         <v>1</v>
       </c>
       <c r="T149" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U149" s="5"/>
       <c r="V149" s="5"/>
@@ -17032,7 +17356,7 @@
         <v>1</v>
       </c>
       <c r="T150" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U150" s="5"/>
       <c r="V150" s="5"/>
@@ -17104,7 +17428,7 @@
         <v>1</v>
       </c>
       <c r="T151" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U151" s="5"/>
       <c r="V151" s="5"/>
@@ -17176,7 +17500,7 @@
         <v>1</v>
       </c>
       <c r="T152" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U152" s="5"/>
       <c r="V152" s="5"/>
@@ -17248,7 +17572,7 @@
         <v>1</v>
       </c>
       <c r="T153" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U153" s="5"/>
       <c r="V153" s="5"/>
@@ -17320,7 +17644,7 @@
         <v>1</v>
       </c>
       <c r="T154" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U154" s="5"/>
       <c r="V154" s="5"/>
@@ -17392,7 +17716,7 @@
         <v>1</v>
       </c>
       <c r="T155" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U155" s="5"/>
       <c r="V155" s="5"/>
@@ -17464,7 +17788,7 @@
         <v>1</v>
       </c>
       <c r="T156" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U156" s="5"/>
       <c r="V156" s="5"/>
@@ -17536,7 +17860,7 @@
         <v>1</v>
       </c>
       <c r="T157" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U157" s="5"/>
       <c r="V157" s="5"/>
@@ -17608,7 +17932,7 @@
         <v>1</v>
       </c>
       <c r="T158" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U158" s="5"/>
       <c r="V158" s="5"/>
@@ -17680,7 +18004,7 @@
         <v>1</v>
       </c>
       <c r="T159" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U159" s="5"/>
       <c r="V159" s="5"/>
@@ -17752,7 +18076,7 @@
         <v>1</v>
       </c>
       <c r="T160" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U160" s="5"/>
       <c r="V160" s="5"/>
@@ -17824,7 +18148,7 @@
         <v>1</v>
       </c>
       <c r="T161" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U161" s="5"/>
       <c r="V161" s="5"/>
@@ -17896,7 +18220,7 @@
         <v>1</v>
       </c>
       <c r="T162" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U162" s="5"/>
       <c r="V162" s="5"/>
@@ -17968,7 +18292,7 @@
         <v>1</v>
       </c>
       <c r="T163" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U163" s="5"/>
       <c r="V163" s="5"/>
@@ -18040,7 +18364,7 @@
         <v>1</v>
       </c>
       <c r="T164" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U164" s="5"/>
       <c r="V164" s="5"/>
@@ -18112,7 +18436,7 @@
         <v>1</v>
       </c>
       <c r="T165" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U165" s="5"/>
       <c r="V165" s="5"/>
@@ -18184,7 +18508,7 @@
         <v>1</v>
       </c>
       <c r="T166" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U166" s="5"/>
       <c r="V166" s="5"/>
@@ -18260,7 +18584,7 @@
         <v>1</v>
       </c>
       <c r="T167" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U167" s="5"/>
       <c r="V167" s="5"/>
@@ -18336,7 +18660,7 @@
         <v>1</v>
       </c>
       <c r="T168" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U168" s="5"/>
       <c r="V168" s="5"/>
@@ -18412,7 +18736,7 @@
         <v>1</v>
       </c>
       <c r="T169" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U169" s="5"/>
       <c r="V169" s="5"/>
@@ -18488,7 +18812,7 @@
         <v>1</v>
       </c>
       <c r="T170" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U170" s="5"/>
       <c r="V170" s="5"/>
@@ -18564,7 +18888,7 @@
         <v>1</v>
       </c>
       <c r="T171" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U171" s="5"/>
       <c r="V171" s="5"/>
@@ -18640,7 +18964,7 @@
         <v>1</v>
       </c>
       <c r="T172" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U172" s="5"/>
       <c r="V172" s="5"/>
@@ -18716,7 +19040,7 @@
         <v>1</v>
       </c>
       <c r="T173" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U173" s="5"/>
       <c r="V173" s="5"/>
@@ -19738,7 +20062,7 @@
         <v>1</v>
       </c>
       <c r="T186" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U186" s="5"/>
       <c r="V186" s="5"/>
@@ -19814,7 +20138,7 @@
         <v>1</v>
       </c>
       <c r="T187" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U187" s="5"/>
       <c r="V187" s="5"/>
@@ -19886,7 +20210,7 @@
         <v>1</v>
       </c>
       <c r="T188" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U188" s="5"/>
       <c r="V188" s="5"/>
@@ -19958,7 +20282,7 @@
         <v>1</v>
       </c>
       <c r="T189" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U189" s="5"/>
       <c r="V189" s="5"/>
@@ -20030,7 +20354,7 @@
         <v>1</v>
       </c>
       <c r="T190" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U190" s="5"/>
       <c r="V190" s="5"/>
@@ -20102,7 +20426,7 @@
         <v>1</v>
       </c>
       <c r="T191" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U191" s="5"/>
       <c r="V191" s="5"/>
@@ -20174,7 +20498,7 @@
         <v>1</v>
       </c>
       <c r="T192" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U192" s="5"/>
       <c r="V192" s="5"/>
@@ -20246,7 +20570,7 @@
         <v>1</v>
       </c>
       <c r="T193" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U193" s="5"/>
       <c r="V193" s="5"/>
@@ -20318,7 +20642,7 @@
         <v>1</v>
       </c>
       <c r="T194" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U194" s="5"/>
       <c r="V194" s="5"/>
@@ -20390,7 +20714,7 @@
         <v>1</v>
       </c>
       <c r="T195" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U195" s="5"/>
       <c r="V195" s="5"/>
@@ -20462,7 +20786,7 @@
         <v>1</v>
       </c>
       <c r="T196" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U196" s="5"/>
       <c r="V196" s="5"/>
@@ -20534,7 +20858,7 @@
         <v>1</v>
       </c>
       <c r="T197" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U197" s="5"/>
       <c r="V197" s="5"/>
@@ -20606,7 +20930,7 @@
         <v>1</v>
       </c>
       <c r="T198" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U198" s="5"/>
       <c r="V198" s="5"/>
@@ -20678,7 +21002,7 @@
         <v>1</v>
       </c>
       <c r="T199" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U199" s="5"/>
       <c r="V199" s="5"/>
@@ -20750,7 +21074,7 @@
         <v>1</v>
       </c>
       <c r="T200" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U200" s="5"/>
       <c r="V200" s="5"/>
@@ -20822,7 +21146,7 @@
         <v>1</v>
       </c>
       <c r="T201" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U201" s="5"/>
       <c r="V201" s="5"/>
@@ -20894,7 +21218,7 @@
         <v>1</v>
       </c>
       <c r="T202" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U202" s="5"/>
       <c r="V202" s="5"/>
@@ -20966,7 +21290,7 @@
         <v>1</v>
       </c>
       <c r="T203" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U203" s="5"/>
       <c r="V203" s="5"/>
@@ -21038,7 +21362,7 @@
         <v>1</v>
       </c>
       <c r="T204" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U204" s="5"/>
       <c r="V204" s="5"/>
@@ -21418,7 +21742,7 @@
         <v>1</v>
       </c>
       <c r="T209" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U209" s="5"/>
       <c r="V209" s="5"/>
@@ -21494,7 +21818,7 @@
         <v>1</v>
       </c>
       <c r="T210" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U210" s="5"/>
       <c r="V210" s="5"/>
@@ -21566,7 +21890,7 @@
         <v>1</v>
       </c>
       <c r="T211" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U211" s="5"/>
       <c r="V211" s="5"/>
@@ -21638,7 +21962,7 @@
         <v>1</v>
       </c>
       <c r="T212" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U212" s="5"/>
       <c r="V212" s="5"/>
@@ -21710,7 +22034,7 @@
         <v>1</v>
       </c>
       <c r="T213" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U213" s="5"/>
       <c r="V213" s="5"/>
@@ -21782,7 +22106,7 @@
         <v>1</v>
       </c>
       <c r="T214" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U214" s="5"/>
       <c r="V214" s="5"/>
@@ -21854,7 +22178,7 @@
         <v>1</v>
       </c>
       <c r="T215" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U215" s="5"/>
       <c r="V215" s="5"/>
@@ -21926,7 +22250,7 @@
         <v>1</v>
       </c>
       <c r="T216" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U216" s="5"/>
       <c r="V216" s="5"/>
@@ -21998,7 +22322,7 @@
         <v>1</v>
       </c>
       <c r="T217" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U217" s="5"/>
       <c r="V217" s="5"/>
@@ -22070,7 +22394,7 @@
         <v>1</v>
       </c>
       <c r="T218" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U218" s="5"/>
       <c r="V218" s="5"/>
@@ -22455,7 +22779,7 @@
         <v>1</v>
       </c>
       <c r="T223" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U223" s="5"/>
       <c r="V223" s="5"/>
@@ -22531,7 +22855,7 @@
         <v>1</v>
       </c>
       <c r="T224" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U224" s="5"/>
       <c r="V224" s="5"/>
@@ -22607,7 +22931,7 @@
         <v>1</v>
       </c>
       <c r="T225" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U225" s="5"/>
       <c r="V225" s="5"/>
@@ -22683,7 +23007,7 @@
         <v>1</v>
       </c>
       <c r="T226" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U226" s="5"/>
       <c r="V226" s="5"/>
@@ -22755,7 +23079,7 @@
         <v>1</v>
       </c>
       <c r="T227" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U227" s="5"/>
       <c r="V227" s="5"/>
@@ -22827,7 +23151,7 @@
         <v>1</v>
       </c>
       <c r="T228" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U228" s="5"/>
       <c r="V228" s="5"/>
@@ -22899,7 +23223,7 @@
         <v>1</v>
       </c>
       <c r="T229" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U229" s="5"/>
       <c r="V229" s="5"/>
@@ -22971,7 +23295,7 @@
         <v>1</v>
       </c>
       <c r="T230" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U230" s="5"/>
       <c r="V230" s="5"/>
@@ -23043,7 +23367,7 @@
         <v>1</v>
       </c>
       <c r="T231" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U231" s="5"/>
       <c r="V231" s="5"/>
@@ -23115,7 +23439,7 @@
         <v>1</v>
       </c>
       <c r="T232" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U232" s="5"/>
       <c r="V232" s="5"/>
@@ -23187,7 +23511,7 @@
         <v>1</v>
       </c>
       <c r="T233" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U233" s="5"/>
       <c r="V233" s="5"/>
@@ -23259,7 +23583,7 @@
         <v>1</v>
       </c>
       <c r="T234" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U234" s="5"/>
       <c r="V234" s="5"/>
@@ -23331,7 +23655,7 @@
         <v>1</v>
       </c>
       <c r="T235" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U235" s="5"/>
       <c r="V235" s="5"/>
@@ -23404,7 +23728,7 @@
         <v>1</v>
       </c>
       <c r="T236" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U236" s="5"/>
       <c r="V236" s="5"/>
@@ -23476,7 +23800,7 @@
         <v>1</v>
       </c>
       <c r="T237" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U237" s="5"/>
       <c r="V237" s="5"/>
@@ -23548,7 +23872,7 @@
         <v>1</v>
       </c>
       <c r="T238" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U238" s="5"/>
       <c r="V238" s="5"/>
@@ -24535,7 +24859,7 @@
         <v>1</v>
       </c>
       <c r="T251" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U251" s="5"/>
       <c r="V251" s="5"/>
@@ -24607,7 +24931,7 @@
         <v>1</v>
       </c>
       <c r="T252" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U252" s="5"/>
       <c r="V252" s="5"/>
@@ -24679,7 +25003,7 @@
         <v>1</v>
       </c>
       <c r="T253" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U253" s="5"/>
       <c r="V253" s="5"/>
@@ -24751,7 +25075,7 @@
         <v>1</v>
       </c>
       <c r="T254" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U254" s="5"/>
       <c r="V254" s="5"/>
@@ -24823,7 +25147,7 @@
         <v>1</v>
       </c>
       <c r="T255" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U255" s="5"/>
       <c r="V255" s="5"/>
@@ -24895,7 +25219,7 @@
         <v>1</v>
       </c>
       <c r="T256" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U256" s="5"/>
       <c r="V256" s="5"/>
@@ -24967,7 +25291,7 @@
         <v>1</v>
       </c>
       <c r="T257" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U257" s="5"/>
       <c r="V257" s="5"/>
@@ -25039,7 +25363,7 @@
         <v>1</v>
       </c>
       <c r="T258" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U258" s="5"/>
       <c r="V258" s="5"/>
@@ -25111,7 +25435,7 @@
         <v>1</v>
       </c>
       <c r="T259" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U259" s="5"/>
       <c r="V259" s="5"/>
@@ -25183,7 +25507,7 @@
         <v>1</v>
       </c>
       <c r="T260" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U260" s="5"/>
       <c r="V260" s="5"/>
@@ -25255,7 +25579,7 @@
         <v>1</v>
       </c>
       <c r="T261" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U261" s="5"/>
       <c r="V261" s="5"/>
@@ -25327,7 +25651,7 @@
         <v>1</v>
       </c>
       <c r="T262" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U262" s="5"/>
       <c r="V262" s="5"/>
@@ -25399,7 +25723,7 @@
         <v>1</v>
       </c>
       <c r="T263" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U263" s="5"/>
       <c r="V263" s="5"/>
@@ -25475,7 +25799,7 @@
         <v>1</v>
       </c>
       <c r="T264" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U264" s="5"/>
       <c r="V264" s="5"/>
@@ -25551,7 +25875,7 @@
         <v>1</v>
       </c>
       <c r="T265" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U265" s="5"/>
       <c r="V265" s="5"/>
@@ -25627,7 +25951,7 @@
         <v>1</v>
       </c>
       <c r="T266" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U266" s="5"/>
       <c r="V266" s="5"/>
@@ -25778,7 +26102,7 @@
         <v>1</v>
       </c>
       <c r="T268" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U268" s="5"/>
       <c r="V268" s="5"/>
@@ -25854,7 +26178,7 @@
         <v>1</v>
       </c>
       <c r="T269" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U269" s="5"/>
       <c r="V269" s="5"/>
@@ -25930,7 +26254,7 @@
         <v>1</v>
       </c>
       <c r="T270" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U270" s="5"/>
       <c r="V270" s="5"/>
@@ -26006,7 +26330,7 @@
         <v>1</v>
       </c>
       <c r="T271" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U271" s="5"/>
       <c r="V271" s="5"/>
@@ -26082,7 +26406,7 @@
         <v>1</v>
       </c>
       <c r="T272" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U272" s="5"/>
       <c r="V272" s="5"/>
@@ -26158,7 +26482,7 @@
         <v>1</v>
       </c>
       <c r="T273" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U273" s="5"/>
       <c r="V273" s="5"/>
@@ -26310,7 +26634,7 @@
         <v>1</v>
       </c>
       <c r="T275" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U275" s="5"/>
       <c r="V275" s="5"/>
@@ -26382,7 +26706,7 @@
         <v>1</v>
       </c>
       <c r="T276" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U276" s="5"/>
       <c r="V276" s="5"/>
@@ -26454,7 +26778,7 @@
         <v>1</v>
       </c>
       <c r="T277" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U277" s="5"/>
       <c r="V277" s="5"/>
@@ -26526,7 +26850,7 @@
         <v>1</v>
       </c>
       <c r="T278" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U278" s="5"/>
       <c r="V278" s="5"/>
@@ -26598,7 +26922,7 @@
         <v>1</v>
       </c>
       <c r="T279" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U279" s="5"/>
       <c r="V279" s="5"/>
@@ -26670,7 +26994,7 @@
         <v>1</v>
       </c>
       <c r="T280" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U280" s="5"/>
       <c r="V280" s="5"/>
@@ -26742,7 +27066,7 @@
         <v>1</v>
       </c>
       <c r="T281" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U281" s="5"/>
       <c r="V281" s="5"/>
@@ -26818,7 +27142,7 @@
         <v>1</v>
       </c>
       <c r="T282" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U282" s="5"/>
       <c r="V282" s="5"/>
@@ -26890,7 +27214,7 @@
         <v>1</v>
       </c>
       <c r="T283" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U283" s="5"/>
       <c r="V283" s="5"/>
@@ -26962,7 +27286,7 @@
         <v>1</v>
       </c>
       <c r="T284" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U284" s="5"/>
       <c r="V284" s="5"/>
@@ -27034,7 +27358,7 @@
         <v>1</v>
       </c>
       <c r="T285" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U285" s="5"/>
       <c r="V285" s="5"/>
@@ -27106,7 +27430,7 @@
         <v>1</v>
       </c>
       <c r="T286" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U286" s="5"/>
       <c r="V286" s="5"/>
@@ -27178,7 +27502,7 @@
         <v>1</v>
       </c>
       <c r="T287" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U287" s="5"/>
       <c r="V287" s="5"/>
@@ -27250,7 +27574,7 @@
         <v>1</v>
       </c>
       <c r="T288" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U288" s="5"/>
       <c r="V288" s="5"/>
@@ -27322,7 +27646,7 @@
         <v>1</v>
       </c>
       <c r="T289" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U289" s="5"/>
       <c r="V289" s="5"/>
@@ -27394,7 +27718,7 @@
         <v>1</v>
       </c>
       <c r="T290" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U290" s="5"/>
       <c r="V290" s="5"/>
@@ -27466,7 +27790,7 @@
         <v>1</v>
       </c>
       <c r="T291" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U291" s="5"/>
       <c r="V291" s="5"/>
@@ -27610,7 +27934,7 @@
         <v>1</v>
       </c>
       <c r="T293" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U293" s="5"/>
       <c r="V293" s="5"/>
@@ -27682,7 +28006,7 @@
         <v>1</v>
       </c>
       <c r="T294" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U294" s="5"/>
       <c r="V294" s="5"/>
@@ -27754,7 +28078,7 @@
         <v>1</v>
       </c>
       <c r="T295" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U295" s="5"/>
       <c r="V295" s="5"/>
@@ -27826,7 +28150,7 @@
         <v>1</v>
       </c>
       <c r="T296" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U296" s="5"/>
       <c r="V296" s="5"/>
@@ -27898,7 +28222,7 @@
         <v>1</v>
       </c>
       <c r="T297" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U297" s="5"/>
       <c r="V297" s="5"/>
@@ -27970,7 +28294,7 @@
         <v>1</v>
       </c>
       <c r="T298" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U298" s="5"/>
       <c r="V298" s="5"/>
@@ -28042,7 +28366,7 @@
         <v>1</v>
       </c>
       <c r="T299" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U299" s="5"/>
       <c r="V299" s="5"/>
@@ -28118,7 +28442,7 @@
         <v>1</v>
       </c>
       <c r="T300" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U300" s="5"/>
       <c r="V300" s="5"/>
@@ -28350,7 +28674,7 @@
         <v>1</v>
       </c>
       <c r="T303" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U303" s="5"/>
       <c r="V303" s="5"/>
@@ -28426,7 +28750,7 @@
         <v>1</v>
       </c>
       <c r="T304" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U304" s="5"/>
       <c r="V304" s="5"/>
@@ -30001,7 +30325,7 @@
         <v>87</v>
       </c>
       <c r="J325" s="5">
-        <f t="shared" ref="J325:J388" si="16">SUM(E325:I325)</f>
+        <f t="shared" ref="J325:J351" si="16">SUM(E325:I325)</f>
         <v>439</v>
       </c>
       <c r="K325" s="5">
@@ -31884,7 +32208,7 @@
         <v>1</v>
       </c>
       <c r="T349" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U349" s="5"/>
       <c r="V349" s="5"/>
@@ -32034,7 +32358,7 @@
         <v>1</v>
       </c>
       <c r="T351" s="5" t="s">
-        <v>296</v>
+        <v>989</v>
       </c>
       <c r="U351" s="5"/>
       <c r="V351" s="5"/>
@@ -32064,635 +32388,731 @@
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="H323:I328 E308:I309 H312:I319 E312:G351 E281:I299 H181:I181 E5:I14 E166:F166 F167 F168:I168 E119:F119 E169:F169 E170:I170 E172:I172 E171:F171 E176:G177 E180:G181 E182:F182 E173:F175 E178:F179 E183:I274 E120:I165 H19:I88 E19:G118">
-    <cfRule type="cellIs" dxfId="178" priority="335" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="218" priority="375" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H93:I118 H89:I90">
-    <cfRule type="cellIs" dxfId="177" priority="333" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="217" priority="373" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H330:I330">
-    <cfRule type="cellIs" dxfId="176" priority="331" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="216" priority="371" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H329:I329">
-    <cfRule type="cellIs" dxfId="175" priority="329" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="215" priority="369" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H332:I332">
-    <cfRule type="cellIs" dxfId="174" priority="327" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="214" priority="367" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H333:I333">
-    <cfRule type="cellIs" dxfId="173" priority="322" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="213" priority="362" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H340:I340">
-    <cfRule type="cellIs" dxfId="172" priority="320" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="212" priority="360" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H341:I341">
-    <cfRule type="cellIs" dxfId="171" priority="318" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="211" priority="358" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H342:I342">
-    <cfRule type="cellIs" dxfId="170" priority="316" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="210" priority="356" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H343:I343">
-    <cfRule type="cellIs" dxfId="169" priority="311" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="209" priority="351" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H344:I344">
-    <cfRule type="cellIs" dxfId="168" priority="307" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="208" priority="347" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H345:I345">
-    <cfRule type="cellIs" dxfId="167" priority="303" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="207" priority="343" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H320:I320">
-    <cfRule type="cellIs" dxfId="166" priority="298" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="206" priority="338" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H321:I321">
-    <cfRule type="cellIs" dxfId="165" priority="297" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="205" priority="337" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H346:I346">
-    <cfRule type="cellIs" dxfId="164" priority="296" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="204" priority="336" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H347:I347">
-    <cfRule type="cellIs" dxfId="163" priority="295" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="203" priority="335" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H348:I348">
-    <cfRule type="cellIs" dxfId="162" priority="294" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="202" priority="334" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H334:I334">
-    <cfRule type="cellIs" dxfId="161" priority="293" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="201" priority="333" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H335:I335">
-    <cfRule type="cellIs" dxfId="160" priority="288" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="200" priority="328" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H336:I336">
-    <cfRule type="cellIs" dxfId="159" priority="287" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="199" priority="327" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H337:I337">
-    <cfRule type="cellIs" dxfId="158" priority="286" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="198" priority="326" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H338:I338">
-    <cfRule type="cellIs" dxfId="157" priority="285" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="197" priority="325" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H339:I339">
-    <cfRule type="cellIs" dxfId="156" priority="284" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="196" priority="324" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H322:I322">
-    <cfRule type="cellIs" dxfId="155" priority="277" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="195" priority="317" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H177:I177">
-    <cfRule type="cellIs" dxfId="154" priority="270" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="194" priority="310" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H91:I91">
-    <cfRule type="cellIs" dxfId="153" priority="269" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="193" priority="309" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H349:I349">
-    <cfRule type="cellIs" dxfId="152" priority="260" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="192" priority="300" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H331:I331">
-    <cfRule type="cellIs" dxfId="151" priority="256" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="191" priority="296" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H350:I350">
-    <cfRule type="cellIs" dxfId="150" priority="251" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="190" priority="291" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H351:I351">
-    <cfRule type="cellIs" dxfId="149" priority="241" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="189" priority="281" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H180:I180">
-    <cfRule type="cellIs" dxfId="148" priority="238" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="188" priority="278" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H92:I92">
-    <cfRule type="cellIs" dxfId="147" priority="234" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="187" priority="274" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T1:T14 T308:T309 T312:T1048576 T299 T281 T206:T209 T220:T246 T263:T274 T88:T123 T145:T186 T19:T86">
-    <cfRule type="cellIs" dxfId="146" priority="222" operator="equal">
+  <conditionalFormatting sqref="T308:T309 T312:T348 T206:T208 T220:T222 T267 T88:T119 T1:T17 T19:T86 T145:T185 T239:T246 T274 T350 T352:T1048576">
+    <cfRule type="cellIs" dxfId="186" priority="262" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="223" operator="equal">
+    <cfRule type="cellIs" dxfId="185" priority="263" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="224" operator="equal">
+    <cfRule type="cellIs" dxfId="184" priority="264" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="225" operator="equal">
+    <cfRule type="cellIs" dxfId="183" priority="265" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="226" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="266" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="227" operator="equal">
+    <cfRule type="cellIs" dxfId="181" priority="267" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="228" operator="equal">
+    <cfRule type="cellIs" dxfId="180" priority="268" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="229" operator="equal">
+    <cfRule type="cellIs" dxfId="179" priority="269" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="230" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="270" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="231" operator="equal">
+    <cfRule type="cellIs" dxfId="177" priority="271" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T300:T307">
-    <cfRule type="cellIs" dxfId="136" priority="197" operator="equal">
+  <conditionalFormatting sqref="T301:T302 T305:T307">
+    <cfRule type="cellIs" dxfId="176" priority="237" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="198" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="238" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="134" priority="199" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="239" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="200" operator="equal">
+    <cfRule type="cellIs" dxfId="173" priority="240" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="201" operator="equal">
+    <cfRule type="cellIs" dxfId="172" priority="241" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="202" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="242" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="203" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="243" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="204" operator="equal">
+    <cfRule type="cellIs" dxfId="169" priority="244" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="128" priority="205" operator="equal">
+    <cfRule type="cellIs" dxfId="168" priority="245" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="206" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="246" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T310">
-    <cfRule type="cellIs" dxfId="126" priority="184" operator="equal">
+    <cfRule type="cellIs" dxfId="166" priority="224" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="185" operator="equal">
+    <cfRule type="cellIs" dxfId="165" priority="225" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="226" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="187" operator="equal">
+    <cfRule type="cellIs" dxfId="163" priority="227" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="188" operator="equal">
+    <cfRule type="cellIs" dxfId="162" priority="228" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="189" operator="equal">
+    <cfRule type="cellIs" dxfId="161" priority="229" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="190" operator="equal">
+    <cfRule type="cellIs" dxfId="160" priority="230" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="191" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="231" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="192" operator="equal">
+    <cfRule type="cellIs" dxfId="158" priority="232" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="193" operator="equal">
+    <cfRule type="cellIs" dxfId="157" priority="233" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T311">
-    <cfRule type="cellIs" dxfId="116" priority="171" operator="equal">
+    <cfRule type="cellIs" dxfId="156" priority="211" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="172" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="212" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="173" operator="equal">
+    <cfRule type="cellIs" dxfId="154" priority="213" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="174" operator="equal">
+    <cfRule type="cellIs" dxfId="153" priority="214" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="175" operator="equal">
+    <cfRule type="cellIs" dxfId="152" priority="215" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="176" operator="equal">
+    <cfRule type="cellIs" dxfId="151" priority="216" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="177" operator="equal">
+    <cfRule type="cellIs" dxfId="150" priority="217" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="178" operator="equal">
+    <cfRule type="cellIs" dxfId="149" priority="218" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="179" operator="equal">
+    <cfRule type="cellIs" dxfId="148" priority="219" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="180" operator="equal">
+    <cfRule type="cellIs" dxfId="147" priority="220" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T282:T298">
-    <cfRule type="cellIs" dxfId="106" priority="158" operator="equal">
+  <conditionalFormatting sqref="T292">
+    <cfRule type="cellIs" dxfId="146" priority="198" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="159" operator="equal">
+    <cfRule type="cellIs" dxfId="145" priority="199" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="160" operator="equal">
+    <cfRule type="cellIs" dxfId="144" priority="200" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="161" operator="equal">
+    <cfRule type="cellIs" dxfId="143" priority="201" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="162" operator="equal">
+    <cfRule type="cellIs" dxfId="142" priority="202" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="163" operator="equal">
+    <cfRule type="cellIs" dxfId="141" priority="203" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="164" operator="equal">
+    <cfRule type="cellIs" dxfId="140" priority="204" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="99" priority="165" operator="equal">
+    <cfRule type="cellIs" dxfId="139" priority="205" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="166" operator="equal">
+    <cfRule type="cellIs" dxfId="138" priority="206" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="167" operator="equal">
+    <cfRule type="cellIs" dxfId="137" priority="207" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E275:I280">
-    <cfRule type="cellIs" dxfId="96" priority="157" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="136" priority="197" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T275:T280">
-    <cfRule type="cellIs" dxfId="95" priority="144" operator="equal">
+  <conditionalFormatting sqref="T219">
+    <cfRule type="cellIs" dxfId="125" priority="171" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="145" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="172" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="146" operator="equal">
+    <cfRule type="cellIs" dxfId="123" priority="173" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="147" operator="equal">
+    <cfRule type="cellIs" dxfId="122" priority="174" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="148" operator="equal">
+    <cfRule type="cellIs" dxfId="121" priority="175" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="149" operator="equal">
+    <cfRule type="cellIs" dxfId="120" priority="176" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="150" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="177" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="151" operator="equal">
+    <cfRule type="cellIs" dxfId="118" priority="178" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="152" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="179" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="153" operator="equal">
-      <formula>"帅"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T210:T219">
-    <cfRule type="cellIs" dxfId="85" priority="131" operator="equal">
-      <formula>"炮"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="132" operator="equal">
-      <formula>"弩"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="133" operator="equal">
-      <formula>"弓"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="134" operator="equal">
-      <formula>"医"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="135" operator="equal">
-      <formula>"乐"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="136" operator="equal">
-      <formula>"鼓"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="137" operator="equal">
-      <formula>"相"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="138" operator="equal">
-      <formula>"扇"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="139" operator="equal">
-      <formula>"谋"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="140" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="180" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G166">
-    <cfRule type="cellIs" dxfId="75" priority="115" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="115" priority="155" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H166:I166">
-    <cfRule type="cellIs" dxfId="74" priority="114" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="114" priority="154" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G167:I167">
-    <cfRule type="cellIs" dxfId="73" priority="113" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="113" priority="153" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E167:E168">
-    <cfRule type="cellIs" dxfId="72" priority="112" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="112" priority="152" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G119:I119">
-    <cfRule type="cellIs" dxfId="71" priority="111" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="111" priority="151" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G169:I169">
-    <cfRule type="cellIs" dxfId="70" priority="110" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="110" priority="150" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G171:I171">
-    <cfRule type="cellIs" dxfId="69" priority="109" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="109" priority="149" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G173:I173">
-    <cfRule type="cellIs" dxfId="68" priority="108" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="108" priority="148" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G174:I174">
-    <cfRule type="cellIs" dxfId="67" priority="107" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="107" priority="147" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G178:I178">
-    <cfRule type="cellIs" dxfId="66" priority="95" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="106" priority="135" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H176:I176">
-    <cfRule type="cellIs" dxfId="65" priority="94" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="105" priority="134" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G182:I182">
-    <cfRule type="cellIs" dxfId="64" priority="93" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="104" priority="133" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G175:I175">
-    <cfRule type="cellIs" dxfId="63" priority="92" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="103" priority="132" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G179:I179">
-    <cfRule type="cellIs" dxfId="62" priority="91" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="102" priority="131" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T187:T205">
-    <cfRule type="cellIs" dxfId="61" priority="78" operator="equal">
+  <conditionalFormatting sqref="T205">
+    <cfRule type="cellIs" dxfId="101" priority="118" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="79" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="119" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="120" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="121" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="122" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="123" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="124" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="85" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="125" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="126" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="127" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T247:T262">
-    <cfRule type="cellIs" dxfId="51" priority="68" operator="equal">
+  <conditionalFormatting sqref="T247:T250">
+    <cfRule type="cellIs" dxfId="91" priority="108" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="109" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="70" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="110" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="111" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="112" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="73" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="113" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="114" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="75" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="115" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="116" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="117" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15:I17">
-    <cfRule type="cellIs" dxfId="41" priority="66" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="81" priority="106" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T15:T17">
-    <cfRule type="cellIs" dxfId="40" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="94" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="95" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="96" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="57" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="97" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="58" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="98" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="59" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="99" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="100" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="101" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="102" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="103" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:I18">
-    <cfRule type="cellIs" dxfId="30" priority="52" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="70" priority="92" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T18">
-    <cfRule type="cellIs" dxfId="29" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="80" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="81" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="82" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="83" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="84" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="85" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="86" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="87" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="88" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="89" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T87">
-    <cfRule type="cellIs" dxfId="19" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="54" operator="equal">
       <formula>"炮"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="55" operator="equal">
       <formula>"弩"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="56" operator="equal">
       <formula>"弓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="57" operator="equal">
       <formula>"医"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="58" operator="equal">
       <formula>"乐"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="59" operator="equal">
       <formula>"鼓"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="60" operator="equal">
       <formula>"相"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="61" operator="equal">
       <formula>"扇"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="62" operator="equal">
       <formula>"谋"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="63" operator="equal">
       <formula>"帅"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T124:T144">
+  <conditionalFormatting sqref="T139:T144">
+    <cfRule type="cellIs" dxfId="49" priority="41" operator="equal">
+      <formula>"炮"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="42" operator="equal">
+      <formula>"弩"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="43" operator="equal">
+      <formula>"弓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="44" operator="equal">
+      <formula>"医"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="45" operator="equal">
+      <formula>"乐"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="44" priority="46" operator="equal">
+      <formula>"鼓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
+      <formula>"相"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="48" operator="equal">
+      <formula>"扇"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="41" priority="49" operator="equal">
+      <formula>"谋"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="50" operator="equal">
+      <formula>"帅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T120:T138">
+    <cfRule type="cellIs" dxfId="39" priority="31" operator="equal">
+      <formula>"炮"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="32" operator="equal">
+      <formula>"弩"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="33" operator="equal">
+      <formula>"弓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="34" operator="equal">
+      <formula>"医"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="35" priority="35" operator="equal">
+      <formula>"乐"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="36" operator="equal">
+      <formula>"鼓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="37" operator="equal">
+      <formula>"相"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="38" operator="equal">
+      <formula>"扇"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="39" operator="equal">
+      <formula>"谋"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="40" operator="equal">
+      <formula>"帅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T209:T218 T186:T204">
+    <cfRule type="cellIs" dxfId="29" priority="21" operator="equal">
+      <formula>"炮"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="22" operator="equal">
+      <formula>"弩"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="23" operator="equal">
+      <formula>"弓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="24" operator="equal">
+      <formula>"医"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="25" operator="equal">
+      <formula>"乐"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="26" operator="equal">
+      <formula>"鼓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="23" priority="27" operator="equal">
+      <formula>"相"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="28" operator="equal">
+      <formula>"扇"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="29" operator="equal">
+      <formula>"谋"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="30" operator="equal">
+      <formula>"帅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T293:T300 T275:T291 T268:T273 T251:T266 T223:T238">
+    <cfRule type="cellIs" dxfId="19" priority="11" operator="equal">
+      <formula>"炮"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="12" operator="equal">
+      <formula>"弩"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="13" operator="equal">
+      <formula>"弓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="14" operator="equal">
+      <formula>"医"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
+      <formula>"乐"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="16" operator="equal">
+      <formula>"鼓"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="17" operator="equal">
+      <formula>"相"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="18" operator="equal">
+      <formula>"扇"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="19" operator="equal">
+      <formula>"谋"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="20" operator="equal">
+      <formula>"帅"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T351 T349 T303:T304">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"炮"</formula>
     </cfRule>

</xml_diff>